<commit_message>
chore: store departments in the import templates; one-shot fake-product cleanup
- Templates (xlsx, CSV example, AI instructions): the 13 store
  departments (Detersivi … Profumeria) replace the demo categories; the
  Excel "categoria" column only accepts them.
- Home "In evidenza": featured products first, then the rest, so it is
  never empty while no product is marked featured.
- tools/demo: demo-catalog/demo-cleanup replaced by
  delete-fake-products.sql (permanent removal of the hidden placeholder
  products and old categories).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ChxsP36S5FxXgxrebAvN6Z
</commit_message>
<xml_diff>
--- a/apps/admin/public/modello-prodotti-casa-te.xlsx
+++ b/apps/admin/public/modello-prodotti-casa-te.xlsx
@@ -18685,8 +18685,8 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Categoria" prompt="Scegli dal menu o scrivi un nome nuovo" type="list">
-      <formula1>=Categorie!$A$2:$A$20</formula1>
+    <dataValidation sqref="C2:C501" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Reparto" error="Scegli uno dei reparti dal menu" promptTitle="Categoria" prompt="Scegli dal menu o scrivi un nome nuovo" type="list">
+      <formula1>=Categorie!$A$2:$A$14</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G501" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"22,10,5,4,0"</formula1>
@@ -18723,6 +18723,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -18772,6 +18773,7 @@
         </is>
       </c>
     </row>
+    <row r="10"/>
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
@@ -18866,17 +18868,17 @@
       </c>
       <c r="C14" s="9" t="inlineStr">
         <is>
-          <t>大类，从下拉选；写新名字会自动新建大类</t>
+          <t>大类（13个部门之一），从下拉选择：Detersivi / Casalinghi / Tessile / Bagno / Idraulica / Ferramenta / Monouso / Giardinaggio / Stagionale / Pets / Giocattoli / Cartoleria / Profumeria</t>
         </is>
       </c>
       <c r="D14" s="9" t="inlineStr">
         <is>
-          <t>Categoria principale (dal menu; un nome nuovo crea la categoria)</t>
+          <t>Reparto del negozio, dal menu: Detersivi, Casalinghi, Tessile, Bagno, Idraulica, Ferramenta, Monouso, Giardinaggio, Stagionale, Pets, Giocattoli, Cartoleria, Profumeria</t>
         </is>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Tessile</t>
         </is>
       </c>
     </row>
@@ -18899,7 +18901,7 @@
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>Profumatori</t>
+          <t>Tavola</t>
         </is>
       </c>
     </row>
@@ -19800,12 +19802,12 @@
       </c>
       <c r="C2" s="11" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Profumeria</t>
         </is>
       </c>
       <c r="D2" s="11" t="inlineStr">
         <is>
-          <t>Profumatori</t>
+          <t>Profumatori ambiente</t>
         </is>
       </c>
       <c r="E2" s="11" t="inlineStr">
@@ -19915,12 +19917,12 @@
       </c>
       <c r="C3" s="11" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Profumeria</t>
         </is>
       </c>
       <c r="D3" s="11" t="inlineStr">
         <is>
-          <t>Profumatori</t>
+          <t>Profumatori ambiente</t>
         </is>
       </c>
       <c r="E3" s="11" t="inlineStr">
@@ -20014,12 +20016,12 @@
       </c>
       <c r="C4" s="11" t="inlineStr">
         <is>
-          <t>Casa</t>
+          <t>Tessile</t>
         </is>
       </c>
       <c r="D4" s="11" t="inlineStr">
         <is>
-          <t>Tessili</t>
+          <t>Tavola</t>
         </is>
       </c>
       <c r="E4" s="11" t="inlineStr">
@@ -20150,7 +20152,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B8"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -20172,67 +20174,115 @@
     <row r="2">
       <c r="A2" s="14" t="inlineStr">
         <is>
-          <t>Pulizia</t>
-        </is>
-      </c>
-      <c r="B2" s="14" t="inlineStr">
-        <is>
-          <t>Carta e monouso, Accessori pulizia</t>
-        </is>
-      </c>
+          <t>Detersivi</t>
+        </is>
+      </c>
+      <c r="B2" s="14" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="14" t="inlineStr">
         <is>
-          <t>Cucina</t>
-        </is>
-      </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>Pentole e padelle, Conservazione, Stoviglie</t>
-        </is>
-      </c>
+          <t>Casalinghi</t>
+        </is>
+      </c>
+      <c r="B3" s="14" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
-          <t>Casa</t>
-        </is>
-      </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>Illuminazione, Decorazione, Tessili</t>
-        </is>
-      </c>
+          <t>Tessile</t>
+        </is>
+      </c>
+      <c r="B4" s="14" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="14" t="inlineStr">
         <is>
-          <t>Detersivo</t>
-        </is>
-      </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>Lavatrice</t>
-        </is>
-      </c>
+          <t>Bagno</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>Organizzazione</t>
-        </is>
-      </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>Scatole e contenitori, Pattumiere</t>
-        </is>
-      </c>
+          <t>Idraulica</t>
+        </is>
+      </c>
+      <c r="B6" s="14" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="14" t="inlineStr">
+        <is>
+          <t>Ferramenta</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="15" t="inlineStr">
-        <is>
-          <t>Puoi usare anche categorie o sottocategorie nuove: vengono create durante l'importazione. / 也可以填新的大类或子类，导入时会自动创建。</t>
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>Monouso</t>
+        </is>
+      </c>
+      <c r="B8" s="14" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Giardinaggio</t>
+        </is>
+      </c>
+      <c r="B9" s="14" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>Stagionale</t>
+        </is>
+      </c>
+      <c r="B10" s="14" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>Pets</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Cibo gatto, Cibo cane, Accessori</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Giocattoli</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="14" t="inlineStr">
+        <is>
+          <t>Cartoleria</t>
+        </is>
+      </c>
+      <c r="B13" s="14" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>Profumeria</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="15" t="inlineStr">
+        <is>
+          <t>Usa uno di questi reparti. Le sottocategorie sono facoltative: un nome nuovo viene creato sotto il reparto. / 请从这13个大类中选；子类可选，写新名字会自动创建。</t>
         </is>
       </c>
     </row>

</xml_diff>